<commit_message>
data: hourly update 2026-07-17 16:26Z
</commit_message>
<xml_diff>
--- a/sports_wagering_pipeline/data/output/latest.xlsx
+++ b/sports_wagering_pipeline/data/output/latest.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>generated 2026-07-16T15:09:04  |  slate 2026-07-16  |  source: shared</t>
+          <t>generated 2026-07-17T16:26:35  |  slate 2026-07-17  |  source: shared</t>
         </is>
       </c>
     </row>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5 (Total)</t>
+          <t>Under 10.5 (Total)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>31.2% EV</t>
+          <t>34.9% EV</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -963,7 +963,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -973,21 +973,21 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 10.5</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.6559</v>
+        <v>0.6077</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.3118</v>
+        <v>0.3491</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T00:10:00Z</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1009,21 +1009,21 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.6299</v>
+        <v>0.5788</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.2598</v>
+        <v>0.2878</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T17:35:00Z</t>
+          <t>2026-07-17T23:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1045,33 +1045,33 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.6077</v>
+        <v>0.6122</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.2458</v>
+        <v>0.2489</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-17T23:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Portland Fire @ Washington Mystics</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1081,21 +1081,21 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>104</v>
+        <v>144</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.7226</v>
+        <v>0.5557</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.2371</v>
+        <v>0.2306</v>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16T23:00Z</t>
+          <t>2026-07-17T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1107,43 +1107,43 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Colorado Rockies</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.598</v>
+        <v>0.6119</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.196</v>
+        <v>0.2183</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-07-17T23:15:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1153,21 +1153,21 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Over 163.5</t>
+          <t>Under 11.0</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>-106</v>
+        <v>113</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.6623</v>
+        <v>0.6034</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.1364</v>
+        <v>0.1979</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T02:00Z</t>
+          <t>2026-07-18T00:05:00Z</t>
         </is>
       </c>
     </row>
@@ -1179,43 +1179,43 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
+          <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Toronto Tempo +6.5</t>
+          <t>Over 174.5</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.5998</v>
+        <v>0.6974</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.1273</v>
+        <v>0.1888</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Portland Fire @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1225,21 +1225,21 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 172.5</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.4813</v>
+        <v>0.6848</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.0877</v>
+        <v>0.18</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16T23:10:00Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
@@ -1251,31 +1251,31 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Over 183.5</t>
+          <t>Indiana Fever +1.5</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-105</v>
+        <v>104</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.5855</v>
+        <v>0.6609</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.0703</v>
+        <v>0.1729</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1287,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>New York Liberty @ Dallas Wings</t>
+          <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1297,57 +1297,57 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Dallas Wings</t>
+          <t>Indiana Fever</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>-115</v>
+        <v>117</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.6241</v>
+        <v>0.6168</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.0683</v>
+        <v>0.1588</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T01:00Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Connecticut Sun @ Phoenix Mercury</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Connecticut Sun +5.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.5414</v>
+        <v>0.525</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0.0678</v>
+        <v>0.1553</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2026-07-18T02:00Z</t>
+          <t>2026-07-17T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1369,21 +1369,21 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>-108</v>
+        <v>122</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.6262</v>
+        <v>0.5188</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.0598</v>
+        <v>0.1517</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
@@ -1395,103 +1395,103 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Houston Astros</t>
+          <t>Over 9.0</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.5042</v>
+        <v>0.475</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.0582</v>
+        <v>0.1465</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-17T23:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Chicago Sky</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>-113</v>
+        <v>105</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.5542</v>
+        <v>0.551</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.0482</v>
+        <v>0.1297</v>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-17T23:40:00Z</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Seattle Storm @ Indiana Fever</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Over 177.0</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.487</v>
+        <v>0.59</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.0468</v>
+        <v>0.1063</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-17T23:30Z</t>
         </is>
       </c>
     </row>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1513,21 +1513,21 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Miami Marlins</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>156</v>
+        <v>104</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.4804</v>
+        <v>0.5792</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.0411</v>
+        <v>0.1044</v>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:40:00Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1549,21 +1549,21 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.5187</v>
+        <v>0.5154</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.0374</v>
+        <v>0.0978</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2026-07-16T23:10:00Z</t>
+          <t>2026-07-17T23:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1575,67 +1575,535 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Indiana Fever -10.5</t>
+          <t>Over 149.5</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>108</v>
+        <v>-104</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.5041</v>
+        <v>0.6188</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.029</v>
+        <v>0.0961</v>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-19T00:30Z</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Over 9.5</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>127</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>0.4812</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>0.09229999999999999</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:05:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles @ Houston Astros</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Over 9.0</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>0.4733</v>
+      </c>
+      <c r="G24" s="10" t="n">
+        <v>0.0858</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Over 9.0</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0.4443</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>0.07779999999999999</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-07-17T17:35:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Padres @ Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>0.5164</v>
+      </c>
+      <c r="G26" s="10" t="n">
+        <v>0.0659</v>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Texas Rangers @ Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Over 8.5</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0.4846</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>0.0564</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:15:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
           <t>WNBA</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Atlanta Dream @ Toronto Tempo</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Portland Fire @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Portland Fire +12.5</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>0.5119</v>
+      </c>
+      <c r="G28" s="10" t="n">
+        <v>0.0533</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Chicago Sky</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>-113</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>0.5542</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>108</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>0.5998</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>0.0481</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:07:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>104</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0.5764</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>0.0478</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>New York Mets @ Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>-170</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>0.615</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:05:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles @ Houston Astros</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Houston Astros</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>-108</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0.5495</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>0.0382</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Padres @ Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>0.4621</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0.0333</v>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Over 183.5</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>104</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>0.5134</v>
-      </c>
-      <c r="G23" s="7" t="n">
-        <v>0.0224</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:30Z</t>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Over 9.0</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>123</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0.4212</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>0.0257</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:15:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Minnesota Twins @ Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Minnesota Twins</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>0.4633</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1734,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:26</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1749,7 +2217,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:26</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1764,7 +2232,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1779,7 +2247,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -1794,7 +2262,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1809,7 +2277,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1824,7 +2292,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:56</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1839,7 +2307,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1854,7 +2322,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1869,7 +2337,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:27</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1884,7 +2352,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1899,7 +2367,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1914,7 +2382,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:57</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1929,7 +2397,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1944,7 +2412,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1959,7 +2427,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1974,7 +2442,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1989,7 +2457,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2004,7 +2472,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:28</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2019,7 +2487,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2034,7 +2502,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:58</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2049,7 +2517,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2064,7 +2532,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2079,7 +2547,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2094,7 +2562,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2109,7 +2577,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2124,7 +2592,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:29</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2139,7 +2607,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:30</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2154,7 +2622,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2169,7 +2637,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:08:59</t>
+          <t>2026-07-17 16:26:30</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2184,7 +2652,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:00</t>
+          <t>2026-07-17 16:26:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2199,7 +2667,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:00</t>
+          <t>2026-07-17 16:26:30</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2214,7 +2682,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:00</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2229,7 +2697,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:00</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2244,7 +2712,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:00</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2259,7 +2727,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2274,7 +2742,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2289,7 +2757,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:31</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2304,7 +2772,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2319,7 +2787,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2334,7 +2802,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2349,7 +2817,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2364,7 +2832,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:01</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2379,7 +2847,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2394,7 +2862,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2409,7 +2877,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:32</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2424,7 +2892,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2439,7 +2907,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2454,7 +2922,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2469,7 +2937,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -2484,7 +2952,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2499,7 +2967,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:02</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -2514,7 +2982,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2529,7 +2997,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:33</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2544,7 +3012,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2559,7 +3027,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2574,7 +3042,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2589,7 +3057,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -2604,7 +3072,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2619,7 +3087,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:03</t>
+          <t>2026-07-17 16:26:34</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -2634,7 +3102,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:04</t>
+          <t>2026-07-17 16:26:35</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2649,7 +3117,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:04</t>
+          <t>2026-07-17 16:26:35</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -2664,7 +3132,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:04</t>
+          <t>2026-07-17 16:26:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2679,7 +3147,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:04</t>
+          <t>2026-07-17 16:26:35</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -2694,7 +3162,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-16 15:09:04</t>
+          <t>2026-07-17 16:26:35</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">

</xml_diff>

<commit_message>
data: hourly update 2026-07-17 22:09Z
</commit_message>
<xml_diff>
--- a/sports_wagering_pipeline/data/output/latest.xlsx
+++ b/sports_wagering_pipeline/data/output/latest.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>generated 2026-07-17T18:15:59  |  slate 2026-07-17  |  source: shared</t>
+          <t>generated 2026-07-17T22:09:45  |  slate 2026-07-17  |  source: shared</t>
         </is>
       </c>
     </row>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Colorado Rockies ML (Moneyline)</t>
+          <t>Over 147.5 (Total)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>14.9% EV</t>
+          <t>14.6% EV</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -964,74 +964,74 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Colorado Rockies ML</t>
+          <t>Over 147.5</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>117</v>
+        <v>-105</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.6008</v>
+        <v>0.6627999999999999</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.1488</v>
+        <v>0.1458</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-19T00:30Z</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Portland Fire @ Minnesota Lynx</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Over 174.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>-105</v>
+        <v>178</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.6419</v>
+        <v>0.4121</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.1359</v>
+        <v>0.1455</v>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:00Z</t>
+          <t>2026-07-17T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1057,92 +1057,92 @@
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5317000000000001</v>
+        <v>0.5286999999999999</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.1324</v>
+        <v>0.1367</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-17T23:15:00Z</t>
+          <t>2026-07-17T23:40:00Z</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Atlanta United FC @ Nashville SC</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>362</v>
+        <v>128</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.274</v>
+        <v>0.498</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.1234</v>
+        <v>0.1356</v>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Atlanta United FC @ Nashville SC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Houston Astros -1.5</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>175</v>
+        <v>362</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.4057</v>
+        <v>0.274</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.1155</v>
+        <v>0.1234</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-18T00:10Z</t>
         </is>
       </c>
     </row>
@@ -1168,13 +1168,13 @@
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.3976</v>
+        <v>0.4016</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.1131</v>
+        <v>0.1164</v>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
@@ -1191,44 +1191,44 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>New York Yankees ML</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>104</v>
+        <v>163</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.5792</v>
+        <v>0.4241</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.1044</v>
+        <v>0.1154</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1238,22 +1238,22 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Over 149.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>-104</v>
+        <v>122</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.6188</v>
+        <v>0.502</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.0961</v>
+        <v>0.1143</v>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:30Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Portland Fire @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1275,34 +1275,34 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Over 182.5</t>
+          <t>Over 175.5</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.6082</v>
+        <v>0.6197</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.0941</v>
+        <v>0.1137</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1312,22 +1312,22 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Over 183.0</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.4812</v>
+        <v>0.5969</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.1107</v>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-17T23:30Z</t>
         </is>
       </c>
     </row>
@@ -1339,32 +1339,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>180</v>
+        <v>117</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.3876</v>
+        <v>0.5119</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0.0854</v>
+        <v>0.1107</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>San Francisco Giants @ Seattle Mariners</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1386,59 +1386,59 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Under 12.5</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>-118</v>
+        <v>100</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.7403</v>
+        <v>0.5495</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.0828</v>
+        <v>0.09909999999999999</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:08:00Z</t>
+          <t>2026-07-18T00:40:00Z</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Seattle Storm @ Indiana Fever</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies ML</t>
+          <t>Over 177.0</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-156</v>
+        <v>-102</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.6119</v>
+        <v>0.59</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.0823</v>
+        <v>0.09810000000000001</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-18T20:05:00Z</t>
+          <t>2026-07-17T23:30Z</t>
         </is>
       </c>
     </row>
@@ -1450,32 +1450,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Over 9.0</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.4733</v>
+        <v>0.4778</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.08110000000000001</v>
+        <v>0.0898</v>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1487,32 +1487,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Cincinnati Reds +1.5</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-110</v>
+        <v>150</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.6401</v>
+        <v>0.4344</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.0702</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T00:40:00Z</t>
         </is>
       </c>
     </row>
@@ -1524,27 +1524,27 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox ML</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.547</v>
+        <v>0.4881</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.0837</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
@@ -1566,27 +1566,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Boston Red Sox ML</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.4802</v>
+        <v>0.5666</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.0659</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1615,10 +1615,10 @@
         <v>108</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.5164</v>
+        <v>0.5152</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.0659</v>
+        <v>0.0653</v>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
@@ -1635,32 +1635,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>New York Yankees ML</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>155</v>
+        <v>105</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.4755</v>
+        <v>0.5654</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.0605</v>
+        <v>0.0649</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
@@ -1672,32 +1672,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Chicago Sky ML</t>
+          <t>Golden State Valkyries -8.5</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>-113</v>
+        <v>-105</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.5542</v>
+        <v>0.5663</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.056</v>
+        <v>0.0621</v>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-19T00:30Z</t>
         </is>
       </c>
     </row>
@@ -1709,69 +1709,69 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0.5764</v>
+        <v>0.4863</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>0.0478</v>
+        <v>0.0552</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-17T23:15:00Z</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Golden State Valkyries -8.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>-110</v>
+        <v>105</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.5663</v>
+        <v>0.5137</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>0.0439</v>
+        <v>0.0532</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:30Z</t>
+          <t>2026-07-17T23:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1783,32 +1783,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>New York Yankees +1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-156</v>
+        <v>104</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0.6897</v>
+        <v>0.514</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>0.0422</v>
+        <v>0.0485</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1830,22 +1830,22 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Over 8.0</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>-104</v>
+        <v>122</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.5377999999999999</v>
+        <v>0.4713</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>0.0385</v>
+        <v>0.0463</v>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-17T23:40:00Z</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1867,22 +1867,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Houston Astros ML</t>
+          <t>Chicago White Sox ML</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0.5495</v>
+        <v>0.6006</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0.0382</v>
+        <v>0.0462</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1904,22 +1904,22 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox ML</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.5998</v>
+        <v>0.5679</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0.0334</v>
+        <v>0.0458</v>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1931,69 +1931,69 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Kansas City Royals ML</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>0.4621</v>
+        <v>0.486</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>0.0333</v>
+        <v>0.045</v>
       </c>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Chicago Sky ML</t>
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>115</v>
+        <v>-117</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.5266999999999999</v>
+        <v>0.5542</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>0.0321</v>
+        <v>0.0449</v>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-17T23:30Z</t>
         </is>
       </c>
     </row>
@@ -2010,27 +2010,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>155</v>
+        <v>115</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>0.4047</v>
+        <v>0.4851</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>0.0319</v>
+        <v>0.043</v>
       </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-17T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -2042,44 +2042,44 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers +1.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>-110</v>
+        <v>100</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.5653</v>
+        <v>0.5508999999999999</v>
       </c>
       <c r="G34" s="10" t="n">
-        <v>0.0292</v>
+        <v>0.0421</v>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:15:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2089,59 +2089,59 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Chicago Sky -2</t>
+          <t>New York Yankees +1.5</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>106</v>
+        <v>-150</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>0.4915</v>
+        <v>0.6712</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0.0291</v>
+        <v>0.0415</v>
       </c>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-17T23:05:00Z</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Portland Fire @ Minnesota Lynx</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Portland Fire +13.5</t>
+          <t>Houston Astros ML</t>
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>-104</v>
+        <v>-108</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.5433</v>
+        <v>0.5669</v>
       </c>
       <c r="G36" s="10" t="n">
-        <v>0.028</v>
+        <v>0.0412</v>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:00Z</t>
+          <t>2026-07-18T00:10:00Z</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2167,55 +2167,55 @@
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>0.575</v>
+        <v>0.5411</v>
       </c>
       <c r="G37" s="7" t="n">
-        <v>0.0236</v>
+        <v>0.0352</v>
       </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Portland Fire @ Minnesota Lynx</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Braves ML</t>
+          <t>Portland Fire +13.5</t>
         </is>
       </c>
       <c r="E38" s="8" t="n">
-        <v>-112</v>
+        <v>-104</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>0.5093</v>
+        <v>0.5433</v>
       </c>
       <c r="G38" s="10" t="n">
-        <v>0.0209</v>
+        <v>0.0328</v>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
@@ -2227,36 +2227,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Arizona Diamondbacks ML</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>144</v>
+        <v>-108</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>0.5198</v>
+        <v>0.4909</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>0.2684</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0307</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2264,7 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2278,67 +2274,59 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
-        <v>104</v>
+        <v>-104</v>
       </c>
       <c r="F40" s="9" t="n">
-        <v>0.6093</v>
+        <v>0.5617</v>
       </c>
       <c r="G40" s="10" t="n">
-        <v>0.2431</v>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0293</v>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Los Angeles Sparks @ Chicago Sky</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Under 10.5</t>
+          <t>Chicago Sky -2</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="F41" s="6" t="n">
-        <v>0.6077</v>
+        <v>0.4915</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>0.2276</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0255</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10:00Z</t>
+          <t>2026-07-17T23:30Z</t>
         </is>
       </c>
     </row>
@@ -2350,36 +2338,32 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Texas Rangers +1.5</t>
         </is>
       </c>
       <c r="E42" s="8" t="n">
-        <v>113</v>
+        <v>-108</v>
       </c>
       <c r="F42" s="9" t="n">
-        <v>0.5509999999999999</v>
+        <v>0.5565</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>0.1737</v>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0251</v>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:40:00Z</t>
+          <t>2026-07-17T23:15:00Z</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2375,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2401,17 +2385,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
         <v>125</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>0.5187999999999999</v>
+        <v>0.5746</v>
       </c>
       <c r="G43" s="7" t="n">
-        <v>0.1673</v>
+        <v>0.293</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2420,39 +2404,39 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T23:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>New York Liberty @ Indiana Fever</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Indiana Fever +1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E44" s="8" t="n">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>0.6609</v>
+        <v>0.5956</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>0.1672</v>
+        <v>0.2805</v>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
@@ -2461,19 +2445,19 @@
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>New York Liberty @ Indiana Fever</t>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2483,17 +2467,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>-105</v>
+        <v>117</v>
       </c>
       <c r="F45" s="6" t="n">
-        <v>0.6766</v>
+        <v>0.5843</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>0.1593</v>
+        <v>0.2679</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2502,48 +2486,417 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-07-19T00:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Under 9.5</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>144</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>0.5149</v>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>0.2564</v>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-17T23:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Colorado Rockies ML</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0.6119</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>0.2183</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Minnesota Twins @ Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Under 11.5</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>0.5884</v>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>0.2062</v>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:05:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>WNBA</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Indiana Fever +1.5</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>0.6609</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>0.1909</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles @ Houston Astros</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Houston Astros -1.5</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>175</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="G50" s="10" t="n">
+        <v>0.1788</v>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Baltimore Orioles @ Houston Astros</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Over 8.5</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="n">
+        <v>-111</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>0.6166</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>0.1721</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>New York Liberty @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Moneyline</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>Indiana Fever ML</t>
         </is>
       </c>
-      <c r="E46" s="8" t="n">
-        <v>117</v>
-      </c>
-      <c r="F46" s="9" t="n">
+      <c r="E52" s="8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F52" s="9" t="n">
         <v>0.6168</v>
       </c>
-      <c r="G46" s="10" t="n">
-        <v>0.1588</v>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="G52" s="10" t="n">
+        <v>0.1653</v>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>⚠️ verify news</t>
         </is>
       </c>
-      <c r="I46" s="4" t="inlineStr">
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>New York Liberty @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Over 175.5</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>-108</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>0.6766</v>
+      </c>
+      <c r="G53" s="7" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>San Diego Padres @ Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Under 10.5</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>101</v>
+      </c>
+      <c r="F54" s="9" t="n">
+        <v>0.5736</v>
+      </c>
+      <c r="G54" s="10" t="n">
+        <v>0.1529</v>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Colorado Rockies ML</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="n">
+        <v>-106</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>0.6822</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>0.1508</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-07-18T00:40:00Z</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2995,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:58</t>
+          <t>2026-07-17 22:09:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2657,7 +3010,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:58</t>
+          <t>2026-07-17 22:09:44</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2672,7 +3025,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:58</t>
+          <t>2026-07-17 22:09:44</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2687,7 +3040,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2702,7 +3055,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2717,7 +3070,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -2732,7 +3085,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2747,7 +3100,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2762,7 +3115,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2777,7 +3130,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -2792,7 +3145,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2807,7 +3160,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2822,7 +3175,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2837,7 +3190,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2852,7 +3205,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2867,7 +3220,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2882,7 +3235,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2897,7 +3250,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2912,7 +3265,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2927,7 +3280,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2942,7 +3295,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2957,7 +3310,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2972,7 +3325,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2987,7 +3340,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -3002,7 +3355,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3017,7 +3370,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -3032,7 +3385,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3047,7 +3400,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -3062,7 +3415,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3077,7 +3430,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -3092,7 +3445,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3107,7 +3460,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -3122,7 +3475,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3137,7 +3490,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -3152,7 +3505,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3167,7 +3520,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3182,7 +3535,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3197,7 +3550,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3212,7 +3565,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3227,7 +3580,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3242,7 +3595,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3257,7 +3610,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3272,7 +3625,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3287,7 +3640,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3302,7 +3655,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3317,7 +3670,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3332,7 +3685,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3347,7 +3700,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3362,7 +3715,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3377,7 +3730,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3392,7 +3745,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3407,7 +3760,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3422,7 +3775,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3437,7 +3790,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3452,7 +3805,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3467,7 +3820,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3482,7 +3835,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3497,7 +3850,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3512,7 +3865,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3527,7 +3880,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3542,7 +3895,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3557,7 +3910,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3572,7 +3925,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3587,7 +3940,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -3602,7 +3955,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-17 18:15:59</t>
+          <t>2026-07-17 22:09:45</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">

</xml_diff>

<commit_message>
data: hourly update 2026-07-18 14:30Z
</commit_message>
<xml_diff>
--- a/sports_wagering_pipeline/data/output/latest.xlsx
+++ b/sports_wagering_pipeline/data/output/latest.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>generated 2026-07-17T22:09:45  |  slate 2026-07-17  |  source: shared</t>
+          <t>generated 2026-07-18T14:30:14  |  slate 2026-07-18  |  source: shared</t>
         </is>
       </c>
     </row>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Over 147.5 (Total)</t>
+          <t>Boston Red Sox -1.5 (Spread)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>14.6% EV</t>
+          <t>13.9% EV</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -964,37 +964,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Over 147.5</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-105</v>
+        <v>170</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.6627999999999999</v>
+        <v>0.4219</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.1458</v>
+        <v>0.139</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-19T00:30Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1016,22 +1016,22 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.4121</v>
+        <v>0.4866</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.1455</v>
+        <v>0.1125</v>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1053,22 +1053,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5286999999999999</v>
+        <v>0.5645</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.1367</v>
+        <v>0.1043</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-17T23:40:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1090,34 +1090,34 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.498</v>
+        <v>0.5393</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.1356</v>
+        <v>0.0818</v>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Atlanta United FC @ Nashville SC</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1127,22 +1127,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Colorado Rockies ML</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>362</v>
+        <v>117</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.274</v>
+        <v>0.5288</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.1234</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-18T00:10Z</t>
+          <t>2026-07-19T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1159,27 +1159,27 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Boston Red Sox ML</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>178</v>
+        <v>104</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.4016</v>
+        <v>0.5668</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.1164</v>
+        <v>0.0774</v>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T17:35:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1196,27 +1196,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Boston Red Sox ML</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>163</v>
+        <v>104</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.4241</v>
+        <v>0.545</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.1154</v>
+        <v>0.0774</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1238,34 +1238,34 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
         <v>122</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.502</v>
+        <v>0.4778</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.1143</v>
+        <v>0.0606</v>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T20:05:00Z</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Portland Fire @ Minnesota Lynx</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1275,59 +1275,59 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Over 175.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.6197</v>
+        <v>0.5427</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.1137</v>
+        <v>0.0574</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-19T00:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Over 183.0</t>
+          <t>Colorado Rockies ML</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.5969</v>
+        <v>0.5513</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.1107</v>
+        <v>0.0572</v>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1339,32 +1339,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Kansas City Royals ML</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>117</v>
+        <v>-104</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.5119</v>
+        <v>0.5411</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0.1107</v>
+        <v>0.0547</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1376,69 +1376,69 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Under 12.5</t>
+          <t>Chicago White Sox ML</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.5495</v>
+        <v>0.6051</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.09909999999999999</v>
+        <v>0.054</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T00:40:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Seattle Storm @ Indiana Fever</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Over 177.0</t>
+          <t>Kansas City Royals ML</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-102</v>
+        <v>100</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.59</v>
+        <v>0.5187</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.09810000000000001</v>
+        <v>0.0356</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-17T23:30Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1450,32 +1450,32 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>163</v>
+        <v>117</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.4778</v>
+        <v>0.5433</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.0898</v>
+        <v>0.0356</v>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1487,32 +1487,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Cincinnati Reds +1.5</t>
+          <t>Atlanta Braves ML</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>150</v>
+        <v>-106</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.4344</v>
+        <v>0.5282</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0353</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-18T00:40:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1534,22 +1534,22 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Over 9.0</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.4881</v>
+        <v>0.4573</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.0837</v>
+        <v>0.0338</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1571,22 +1571,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Boston Red Sox ML</t>
+          <t>Miami Marlins ML</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.5666</v>
+        <v>0.4859</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.029</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1598,32 +1598,32 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Kansas City Royals ML</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>108</v>
+        <v>-144</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.5152</v>
+        <v>0.6501</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.0653</v>
+        <v>0.0289</v>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1635,69 +1635,69 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>New York Yankees ML</t>
+          <t>Over 9.0</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.5654</v>
+        <v>0.4607</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.0649</v>
+        <v>0.027</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-07-17T23:05:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Golden State Valkyries -8.5</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>-105</v>
+        <v>-113</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.5663</v>
+        <v>0.6129</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.0621</v>
+        <v>0.025</v>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:30Z</t>
+          <t>2026-07-19T17:40:00Z</t>
         </is>
       </c>
     </row>
@@ -1709,32 +1709,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Toronto Blue Jays ML</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>117</v>
+        <v>-104</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0.4863</v>
+        <v>0.4927</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>0.0552</v>
+        <v>0.0244</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-17T23:15:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1746,32 +1746,32 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Baltimore Orioles -1.5</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.5137</v>
+        <v>0.4093</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>0.0532</v>
+        <v>0.023</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:15:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1783,32 +1783,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Houston Astros ML</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0.514</v>
+        <v>0.4702</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>0.0485</v>
+        <v>0.0203</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-18T18:20:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1830,22 +1830,26 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 7.5</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.4713</v>
+        <v>0.6209</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>0.0463</v>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
+        <v>0.2665</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17T23:40:00Z</t>
+          <t>2026-07-18T17:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1857,32 +1861,36 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chicago White Sox ML</t>
+          <t>Under 13.0</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0.6006</v>
+        <v>0.6246</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0.0462</v>
-      </c>
-      <c r="H29" t="inlineStr"/>
+        <v>0.2123</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1894,44 +1902,48 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.5679</v>
+        <v>0.5092</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0.0458</v>
-      </c>
-      <c r="H30" s="4" t="inlineStr"/>
+        <v>0.1864</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T23:10:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1941,962 +1953,26 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 148.5</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>0.486</v>
+        <v>0.641</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="H31" t="inlineStr"/>
+        <v>0.155</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-07-18T18:20:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Chicago Sky ML</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>-117</v>
-      </c>
-      <c r="F32" s="9" t="n">
-        <v>0.5542</v>
-      </c>
-      <c r="G32" s="10" t="n">
-        <v>0.0449</v>
-      </c>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:30Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Over 9.5</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n">
-        <v>115</v>
-      </c>
-      <c r="F33" s="6" t="n">
-        <v>0.4851</v>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>0.043</v>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Over 8.5</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="n">
-        <v>100</v>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>0.5508999999999999</v>
-      </c>
-      <c r="G34" s="10" t="n">
-        <v>0.0421</v>
-      </c>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Los Angeles Dodgers @ New York Yankees</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>New York Yankees +1.5</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="n">
-        <v>-150</v>
-      </c>
-      <c r="F35" s="6" t="n">
-        <v>0.6712</v>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>0.0415</v>
-      </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:05:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Houston Astros ML</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>-108</v>
-      </c>
-      <c r="F36" s="9" t="n">
-        <v>0.5669</v>
-      </c>
-      <c r="G36" s="10" t="n">
-        <v>0.0412</v>
-      </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Over 8.5</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>0.5411</v>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>0.0352</v>
-      </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2026-07-18T19:07:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Portland Fire @ Minnesota Lynx</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Portland Fire +13.5</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="n">
-        <v>-104</v>
-      </c>
-      <c r="F38" s="9" t="n">
-        <v>0.5433</v>
-      </c>
-      <c r="G38" s="10" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-19T00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Arizona Diamondbacks ML</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n">
-        <v>-108</v>
-      </c>
-      <c r="F39" s="6" t="n">
-        <v>0.4909</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>0.0307</v>
-      </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Over 8.5</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="n">
-        <v>-104</v>
-      </c>
-      <c r="F40" s="9" t="n">
-        <v>0.5617</v>
-      </c>
-      <c r="G40" s="10" t="n">
-        <v>0.0293</v>
-      </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Los Angeles Sparks @ Chicago Sky</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Chicago Sky -2</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="n">
-        <v>105</v>
-      </c>
-      <c r="F41" s="6" t="n">
-        <v>0.4915</v>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>0.0255</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:30Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Texas Rangers +1.5</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="n">
-        <v>-108</v>
-      </c>
-      <c r="F42" s="9" t="n">
-        <v>0.5565</v>
-      </c>
-      <c r="G42" s="10" t="n">
-        <v>0.0251</v>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:15:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Over 7.5</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="n">
-        <v>125</v>
-      </c>
-      <c r="F43" s="6" t="n">
-        <v>0.5746</v>
-      </c>
-      <c r="G43" s="7" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>2026-07-18T23:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Under 9.5</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="n">
-        <v>115</v>
-      </c>
-      <c r="F44" s="9" t="n">
-        <v>0.5956</v>
-      </c>
-      <c r="G44" s="10" t="n">
-        <v>0.2805</v>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>Under 9.5</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="n">
-        <v>117</v>
-      </c>
-      <c r="F45" s="6" t="n">
-        <v>0.5843</v>
-      </c>
-      <c r="G45" s="7" t="n">
-        <v>0.2679</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-07-18T20:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Under 9.5</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="n">
-        <v>144</v>
-      </c>
-      <c r="F46" s="9" t="n">
-        <v>0.5149</v>
-      </c>
-      <c r="G46" s="10" t="n">
-        <v>0.2564</v>
-      </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-17T23:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Colorado Rockies ML</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n">
-        <v>117</v>
-      </c>
-      <c r="F47" s="6" t="n">
-        <v>0.6119</v>
-      </c>
-      <c r="G47" s="7" t="n">
-        <v>0.2183</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>2026-07-18T19:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Under 11.5</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="n">
-        <v>105</v>
-      </c>
-      <c r="F48" s="9" t="n">
-        <v>0.5884</v>
-      </c>
-      <c r="G48" s="10" t="n">
-        <v>0.2062</v>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:05:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Indiana Fever +1.5</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n">
-        <v>108</v>
-      </c>
-      <c r="F49" s="6" t="n">
-        <v>0.6609</v>
-      </c>
-      <c r="G49" s="7" t="n">
-        <v>0.1909</v>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>2026-07-19T00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Spread</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Houston Astros -1.5</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="n">
-        <v>175</v>
-      </c>
-      <c r="F50" s="9" t="n">
-        <v>0.4286</v>
-      </c>
-      <c r="G50" s="10" t="n">
-        <v>0.1788</v>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Over 8.5</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="n">
-        <v>-111</v>
-      </c>
-      <c r="F51" s="6" t="n">
-        <v>0.6166</v>
-      </c>
-      <c r="G51" s="7" t="n">
-        <v>0.1721</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Indiana Fever ML</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="n">
-        <v>120</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>0.6168</v>
-      </c>
-      <c r="G52" s="10" t="n">
-        <v>0.1653</v>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-19T00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>WNBA</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>New York Liberty @ Indiana Fever</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Over 175.5</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="n">
-        <v>-108</v>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>0.6766</v>
-      </c>
-      <c r="G53" s="7" t="n">
-        <v>0.1573</v>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>2026-07-19T00:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Under 10.5</t>
-        </is>
-      </c>
-      <c r="E54" s="8" t="n">
-        <v>101</v>
-      </c>
-      <c r="F54" s="9" t="n">
-        <v>0.5736</v>
-      </c>
-      <c r="G54" s="10" t="n">
-        <v>0.1529</v>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:10:00Z</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>MLB</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Moneyline</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Colorado Rockies ML</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="n">
-        <v>-106</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>0.6822</v>
-      </c>
-      <c r="G55" s="7" t="n">
-        <v>0.1508</v>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>2026-07-18T00:40:00Z</t>
+          <t>2026-07-19T00:30Z</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2071,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:44</t>
+          <t>2026-07-18 14:30:13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3010,7 +2086,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:44</t>
+          <t>2026-07-18 14:30:13</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -3025,7 +2101,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:44</t>
+          <t>2026-07-18 14:30:13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3040,7 +2116,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -3055,7 +2131,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3070,7 +2146,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -3085,7 +2161,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3100,7 +2176,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -3115,7 +2191,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3130,7 +2206,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -3145,7 +2221,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3160,7 +2236,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -3175,7 +2251,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3190,7 +2266,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -3205,7 +2281,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3220,7 +2296,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -3235,7 +2311,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3250,7 +2326,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -3265,7 +2341,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3280,7 +2356,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -3295,7 +2371,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3310,7 +2386,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -3325,7 +2401,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3340,7 +2416,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -3355,7 +2431,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3370,7 +2446,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -3385,7 +2461,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3400,7 +2476,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -3415,7 +2491,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3430,7 +2506,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -3445,7 +2521,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3460,7 +2536,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -3475,7 +2551,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3490,7 +2566,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -3505,7 +2581,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3520,7 +2596,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -3535,7 +2611,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3550,7 +2626,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -3565,7 +2641,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3580,7 +2656,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -3595,7 +2671,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3610,7 +2686,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -3625,7 +2701,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3640,7 +2716,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -3655,7 +2731,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3670,7 +2746,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -3685,7 +2761,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3700,7 +2776,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3715,7 +2791,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3730,7 +2806,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3745,7 +2821,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3760,7 +2836,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3775,7 +2851,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3790,7 +2866,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3805,7 +2881,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3820,7 +2896,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3835,7 +2911,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3850,7 +2926,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3865,7 +2941,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3880,7 +2956,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3895,7 +2971,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3910,7 +2986,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3925,7 +3001,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3940,7 +3016,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -3955,7 +3031,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-17 22:09:45</t>
+          <t>2026-07-18 14:30:14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">

</xml_diff>

<commit_message>
data: hourly update 2026-07-18 18:02Z
</commit_message>
<xml_diff>
--- a/sports_wagering_pipeline/data/output/latest.xlsx
+++ b/sports_wagering_pipeline/data/output/latest.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>generated 2026-07-18T14:30:14  |  slate 2026-07-18  |  source: shared</t>
+          <t>generated 2026-07-18T18:02:21  |  slate 2026-07-18  |  source: shared</t>
         </is>
       </c>
     </row>
@@ -590,16 +590,16 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5 (Spread)</t>
+          <t>Chicago White Sox -1.5 (Spread)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>13.9% EV</t>
+          <t>12.4% EV</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -969,7 +969,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -979,22 +979,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
         <v>170</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.4219</v>
+        <v>0.4946</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.139</v>
+        <v>0.1239</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1011,22 +1011,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>170</v>
+        <v>112</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.4866</v>
+        <v>0.5216000000000001</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.1125</v>
+        <v>0.1058</v>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1053,22 +1053,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Over 8.0</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>113</v>
+        <v>-104</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.5645</v>
+        <v>0.6458</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.1043</v>
+        <v>0.0974</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1090,17 +1090,17 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Over 9.0</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.5393</v>
+        <v>0.4779</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.0818</v>
+        <v>0.0955</v>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
@@ -1131,13 +1131,13 @@
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.5288</v>
+        <v>0.5252</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0829</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
@@ -1159,22 +1159,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox ML</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>104</v>
+        <v>170</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.5668</v>
+        <v>0.3999</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.0774</v>
+        <v>0.07969999999999999</v>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
@@ -1191,32 +1191,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Boston Red Sox ML</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.545</v>
+        <v>0.6008</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.0774</v>
+        <v>0.078</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-19T17:35:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1228,32 +1228,32 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Under 8.5</t>
+          <t>Boston Red Sox ML</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.4778</v>
+        <v>0.5445</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.0606</v>
+        <v>0.0774</v>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:05:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1265,32 +1265,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Colorado Rockies ML</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.5427</v>
+        <v>0.5387999999999999</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.0574</v>
+        <v>0.0644</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1302,32 +1302,32 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Colorado Rockies ML</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>102</v>
+        <v>168</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.5513</v>
+        <v>0.395</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.0572</v>
+        <v>0.0586</v>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1349,22 +1349,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Kansas City Royals ML</t>
+          <t>Chicago White Sox ML</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-104</v>
+        <v>104</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.5411</v>
+        <v>0.6122</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0.0547</v>
+        <v>0.057</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-19T18:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1386,22 +1386,22 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox ML</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.6051</v>
+        <v>0.5462</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.054</v>
+        <v>0.055</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1413,32 +1413,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kansas City Royals ML</t>
+          <t>Over 7.0</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>100</v>
+        <v>-110</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.5187</v>
+        <v>0.5756</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.0356</v>
+        <v>0.0542</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T17:40:00Z</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1460,22 +1460,22 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Philadelphia Phillies ML</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.5433</v>
+        <v>0.4854</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.0356</v>
+        <v>0.053</v>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T23:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1497,17 +1497,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Atlanta Braves ML</t>
+          <t>Kansas City Royals ML</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-106</v>
+        <v>104</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.5282</v>
+        <v>0.5231</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.0353</v>
+        <v>0.0528</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
@@ -1524,32 +1524,32 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Over 9.0</t>
+          <t>Atlanta Braves ML</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>107</v>
+        <v>-104</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.4573</v>
+        <v>0.5312</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.0338</v>
+        <v>0.0463</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Miami Marlins @ Milwaukee Brewers</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1571,22 +1571,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Miami Marlins ML</t>
+          <t>Toronto Blue Jays ML</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>138</v>
+        <v>102</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.4859</v>
+        <v>0.4927</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.029</v>
+        <v>0.0388</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-19T18:10:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1598,32 +1598,32 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Kansas City Royals ML</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>-144</v>
+        <v>-113</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.6501</v>
+        <v>0.5432</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.0289</v>
+        <v>0.0343</v>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1635,32 +1635,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Over 9.0</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>104</v>
+        <v>-138</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.4607</v>
+        <v>0.6355</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.027</v>
+        <v>0.0336</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1682,22 +1682,22 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Houston Astros ML</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>-113</v>
+        <v>100</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.6129</v>
+        <v>0.4823</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.025</v>
+        <v>0.0315</v>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T17:40:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1719,22 +1719,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays ML</t>
+          <t>Minnesota Twins ML</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>-104</v>
+        <v>142</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0.4927</v>
+        <v>0.4799</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>0.0244</v>
+        <v>0.0267</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-19T16:15:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1751,22 +1751,22 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles -1.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>163</v>
+        <v>115</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.4093</v>
+        <v>0.5221</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>0.023</v>
+        <v>0.0222</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1793,22 +1793,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Houston Astros ML</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0.4702</v>
+        <v>0.5291</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>0.0203</v>
+        <v>0.0217</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T17:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1820,36 +1820,32 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>104</v>
+        <v>-125</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.6209</v>
+        <v>0.6309</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>0.2665</v>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0205</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T17:10:00Z</t>
+          <t>2026-07-19T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1861,36 +1857,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Under 13.0</t>
+          <t>Atlanta Braves -1.5</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>106</v>
+        <v>170</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0.6246</v>
+        <v>0.3779</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0.2123</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0202</v>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1894,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -1912,17 +1904,17 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Over 9.5</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.5092</v>
+        <v>0.6054999999999999</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0.1864</v>
+        <v>0.2817</v>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
@@ -1931,48 +1923,253 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T18:20:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Over 7.5</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0.6312</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>0.2751</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Over 7.5</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>0.6278</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0.2682</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T23:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Under 9.5</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0.5647</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>0.1973</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Under 13.0</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>0.6222</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0.1739</v>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>WNBA</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Over 148.5</t>
         </is>
       </c>
-      <c r="E31" s="5" t="n">
-        <v>104</v>
-      </c>
-      <c r="F31" s="6" t="n">
+      <c r="E35" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="F35" s="6" t="n">
         <v>0.641</v>
       </c>
-      <c r="G31" s="7" t="n">
-        <v>0.155</v>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="G35" s="7" t="n">
+        <v>0.1714</v>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>⚠️ verify news</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>2026-07-19T00:30Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>New York Liberty @ Indiana Fever</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Indiana Fever ML</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>0.6189</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0.1588</v>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2268,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:13</t>
+          <t>2026-07-18 18:02:20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2086,7 +2283,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:13</t>
+          <t>2026-07-18 18:02:20</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2101,7 +2298,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:13</t>
+          <t>2026-07-18 18:02:20</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2116,7 +2313,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2131,7 +2328,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2146,7 +2343,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -2161,7 +2358,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2176,7 +2373,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2191,7 +2388,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2206,7 +2403,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -2221,7 +2418,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2236,7 +2433,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2251,7 +2448,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2266,7 +2463,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2281,7 +2478,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2296,7 +2493,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2311,7 +2508,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2326,7 +2523,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2341,7 +2538,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2356,7 +2553,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2371,7 +2568,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2386,7 +2583,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2401,7 +2598,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2416,7 +2613,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2431,7 +2628,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2446,7 +2643,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2461,7 +2658,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2476,7 +2673,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2491,7 +2688,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2506,7 +2703,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2521,7 +2718,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2536,7 +2733,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2551,7 +2748,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2566,7 +2763,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2581,7 +2778,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2596,7 +2793,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2611,7 +2808,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2626,7 +2823,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2641,7 +2838,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2656,7 +2853,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2671,7 +2868,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2686,7 +2883,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2701,7 +2898,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2716,7 +2913,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2731,7 +2928,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2746,7 +2943,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2761,7 +2958,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2776,7 +2973,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -2791,7 +2988,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2806,7 +3003,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -2821,7 +3018,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2836,7 +3033,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -2851,7 +3048,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2866,7 +3063,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2881,7 +3078,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2896,7 +3093,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2911,7 +3108,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2926,7 +3123,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -2941,7 +3138,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2956,7 +3153,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -2971,7 +3168,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2986,7 +3183,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3001,7 +3198,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3016,7 +3213,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -3031,7 +3228,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-18 14:30:14</t>
+          <t>2026-07-18 18:02:21</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">

</xml_diff>

<commit_message>
data: hourly update 2026-07-18 22:04Z
</commit_message>
<xml_diff>
--- a/sports_wagering_pipeline/data/output/latest.xlsx
+++ b/sports_wagering_pipeline/data/output/latest.xlsx
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>generated 2026-07-18T18:14:02  |  slate 2026-07-18  |  source: shared</t>
+          <t>generated 2026-07-18T22:04:26  |  slate 2026-07-18  |  source: shared</t>
         </is>
       </c>
     </row>
@@ -590,11 +590,11 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Under 9.5 (Total)</t>
+          <t>Over 148.5 (Total)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -886,7 +886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -964,12 +964,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Washington Mystics @ Golden State Valkyries</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -979,22 +979,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Over 148.5</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>0.5371</v>
+        <v>0.641</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>0.1387</v>
+        <v>0.1386</v>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-19T00:30Z</t>
         </is>
       </c>
     </row>
@@ -1006,32 +1006,32 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox -1.5</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>170</v>
+        <v>100</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.4874000000000001</v>
+        <v>0.5647</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>0.1171</v>
+        <v>0.1295</v>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1043,32 +1043,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Over 8.0</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-104</v>
+        <v>170</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>0.6458</v>
+        <v>0.4919</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.0974</v>
+        <v>0.1213</v>
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-07-19T18:20:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Over 9.0</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E8" s="8" t="n">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>0.4779</v>
+        <v>0.6503</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>0.0955</v>
+        <v>0.1208</v>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -1117,44 +1117,44 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Colorado Rockies ML</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>0.5288</v>
+        <v>0.5228</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>0.08790000000000001</v>
+        <v>0.1136</v>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-07-19T19:10:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>MLB</t>
+          <t>WNBA</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1164,22 +1164,22 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Connecticut Sun +4.5</t>
         </is>
       </c>
       <c r="E10" s="8" t="n">
-        <v>170</v>
+        <v>106</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>0.3999</v>
+        <v>0.5869</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>0.07969999999999999</v>
+        <v>0.1119</v>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T23:00Z</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1201,22 +1201,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Over 8.5</t>
+          <t>Over 9.0</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0.6008</v>
+        <v>0.4803</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>0.078</v>
+        <v>0.1007</v>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-18T18:20:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1233,27 +1233,27 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox ML</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E12" s="8" t="n">
-        <v>104</v>
+        <v>178</v>
       </c>
       <c r="F12" s="9" t="n">
-        <v>0.5445</v>
+        <v>0.3943</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>0.0774</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1265,32 +1265,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Colorado Rockies ML</t>
+          <t>Boston Red Sox -1.5</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>105</v>
+        <v>170</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>0.5387999999999999</v>
+        <v>0.3999</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>0.0644</v>
+        <v>0.07969999999999999</v>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1302,32 +1302,32 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Boston Red Sox -1.5</t>
+          <t>Pittsburgh Pirates ML</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
-        <v>168</v>
+        <v>122</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>0.3943</v>
+        <v>0.5693</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>0.0567</v>
+        <v>0.0708</v>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T17:35:00Z</t>
+          <t>2026-07-18T23:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1339,32 +1339,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Tampa Bay Rays @ Boston Red Sox</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.5462</v>
+        <v>0.5221</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>0.055</v>
+        <v>0.0702</v>
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-07-18T23:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1376,32 +1376,32 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Over 7.0</t>
+          <t>Philadelphia Phillies ML</t>
         </is>
       </c>
       <c r="E16" s="8" t="n">
-        <v>-110</v>
+        <v>117</v>
       </c>
       <c r="F16" s="9" t="n">
-        <v>0.5756</v>
+        <v>0.4842</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>0.0542</v>
+        <v>0.0696</v>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T17:40:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>San Diego Padres @ Kansas City Royals</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1423,22 +1423,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Kansas City Royals ML</t>
+          <t>Colorado Rockies ML</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.5231</v>
+        <v>0.5479000000000001</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>0.0528</v>
+        <v>0.06850000000000001</v>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1455,27 +1455,27 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Chicago White Sox ML</t>
+          <t>Chicago White Sox -1.5</t>
         </is>
       </c>
       <c r="E18" s="8" t="n">
-        <v>104</v>
+        <v>178</v>
       </c>
       <c r="F18" s="9" t="n">
-        <v>0.6083</v>
+        <v>0.3835</v>
       </c>
       <c r="G18" s="10" t="n">
-        <v>0.0507</v>
+        <v>0.0663</v>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:07:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1487,32 +1487,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>New York Mets @ Philadelphia Phillies</t>
+          <t>Miami Marlins @ Milwaukee Brewers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Philadelphia Phillies ML</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
         <v>108</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>0.4778</v>
+        <v>0.5117</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>0.0504</v>
+        <v>0.06419999999999999</v>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-07-19T17:35:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1524,32 +1524,32 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Braves ML</t>
+          <t>Over 9.5</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>-104</v>
+        <v>122</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.5312</v>
+        <v>0.4762</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.0463</v>
+        <v>0.0572</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1561,32 +1561,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Chicago White Sox @ Toronto Blue Jays</t>
+          <t>New York Mets @ Philadelphia Phillies</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Toronto Blue Jays ML</t>
+          <t>Under 9.0</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>0.4927</v>
+        <v>0.538</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>0.0388</v>
+        <v>0.0565</v>
       </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-07-19T16:15:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1598,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1608,22 +1608,22 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Under 11.5</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
-        <v>-105</v>
+        <v>113</v>
       </c>
       <c r="F22" s="9" t="n">
-        <v>0.5765</v>
+        <v>0.4948</v>
       </c>
       <c r="G22" s="10" t="n">
-        <v>0.0361</v>
+        <v>0.0539</v>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T19:10:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1649,18 +1649,18 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-113</v>
+        <v>104</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0.5411</v>
+        <v>0.5222</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>0.0343</v>
+        <v>0.0532</v>
       </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-07-19T18:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1672,32 +1672,32 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Atlanta Braves ML</t>
         </is>
       </c>
       <c r="E24" s="8" t="n">
-        <v>-138</v>
+        <v>-104</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>0.6355</v>
+        <v>0.5312</v>
       </c>
       <c r="G24" s="10" t="n">
-        <v>0.0336</v>
+        <v>0.0509</v>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-18T20:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1709,32 +1709,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Houston Astros ML</t>
+          <t>Under 9.5</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
         <v>100</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0.4823</v>
+        <v>0.5238</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>0.0315</v>
+        <v>0.0476</v>
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1746,32 +1746,32 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Minnesota Twins @ Chicago Cubs</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Minnesota Twins ML</t>
+          <t>Over 10.5</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
-        <v>142</v>
+        <v>108</v>
       </c>
       <c r="F26" s="9" t="n">
-        <v>0.4799</v>
+        <v>0.5347</v>
       </c>
       <c r="G26" s="10" t="n">
-        <v>0.0267</v>
+        <v>0.0439</v>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T18:20:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1783,32 +1783,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Colorado Rockies +1.5</t>
+          <t>Chicago White Sox ML</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>-125</v>
+        <v>102</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>0.6358</v>
+        <v>0.6086</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>0.0235</v>
+        <v>0.0421</v>
       </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-07-19T19:10:00Z</t>
+          <t>2026-07-18T19:07:00Z</t>
         </is>
       </c>
     </row>
@@ -1820,32 +1820,32 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Baltimore Orioles @ Houston Astros</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Toronto Blue Jays ML</t>
         </is>
       </c>
       <c r="E28" s="8" t="n">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>0.5221</v>
+        <v>0.4927</v>
       </c>
       <c r="G28" s="10" t="n">
-        <v>0.0222</v>
+        <v>0.0394</v>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1857,32 +1857,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Cincinnati Reds @ Colorado Rockies</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Moneyline</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates ML</t>
+          <t>Colorado Rockies +1.5</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>122</v>
+        <v>-138</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0.5291</v>
+        <v>0.6402</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>0.0217</v>
+        <v>0.0365</v>
       </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-07-18T17:10:00Z</t>
+          <t>2026-07-18T19:10:00Z</t>
         </is>
       </c>
     </row>
@@ -1894,32 +1894,32 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Texas Rangers @ Atlanta Braves</t>
+          <t>Chicago White Sox @ Toronto Blue Jays</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Spread</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Atlanta Braves -1.5</t>
+          <t>Under 8.5</t>
         </is>
       </c>
       <c r="E30" s="8" t="n">
-        <v>170</v>
+        <v>105</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>0.3779</v>
+        <v>0.5052</v>
       </c>
       <c r="G30" s="10" t="n">
-        <v>0.0202</v>
+        <v>0.0357</v>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T16:15:00Z</t>
         </is>
       </c>
     </row>
@@ -1931,36 +1931,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Spread</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Under 9.0</t>
+          <t>Pittsburgh Pirates -1.5</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>0.6054999999999999</v>
+        <v>0.4432</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>0.2817</v>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0318</v>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-07-18T20:10:00Z</t>
+          <t>2026-07-19T17:40:00Z</t>
         </is>
       </c>
     </row>
@@ -1972,36 +1968,32 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>Minnesota Twins @ Chicago Cubs</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Minnesota Twins ML</t>
         </is>
       </c>
       <c r="E32" s="8" t="n">
-        <v>102</v>
+        <v>146</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.6312</v>
+        <v>0.4726</v>
       </c>
       <c r="G32" s="10" t="n">
-        <v>0.2751</v>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0296</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18T17:10:00Z</t>
+          <t>2026-07-18T18:20:00Z</t>
         </is>
       </c>
     </row>
@@ -2013,36 +2005,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+          <t>San Diego Padres @ Kansas City Royals</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Over 7.5</t>
+          <t>Kansas City Royals ML</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>102</v>
+        <v>-117</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>0.6278</v>
+        <v>0.5423</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>0.2682</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0268</v>
+      </c>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-07-18T23:10:00Z</t>
+          <t>2026-07-19T18:10:00Z</t>
         </is>
       </c>
     </row>
@@ -2054,33 +2042,29 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays @ Boston Red Sox</t>
+          <t>Baltimore Orioles @ Houston Astros</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Under 9.5</t>
+          <t>Houston Astros ML</t>
         </is>
       </c>
       <c r="E34" s="8" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="F34" s="9" t="n">
-        <v>0.5647</v>
+        <v>0.4752</v>
       </c>
       <c r="G34" s="10" t="n">
-        <v>0.1973</v>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0261</v>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
           <t>2026-07-18T20:10:00Z</t>
@@ -2095,7 +2079,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cincinnati Reds @ Colorado Rockies</t>
+          <t>Texas Rangers @ Atlanta Braves</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2105,108 +2089,703 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Under 13.0</t>
+          <t>Over 8.5</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>0.6222</v>
+        <v>0.5616</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0.1739</v>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.026</v>
+      </c>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-07-18T19:10:00Z</t>
+          <t>2026-07-19T17:35:00Z</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>WNBA</t>
+          <t>MLB</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Washington Mystics @ Golden State Valkyries</t>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Over 148.5</t>
+          <t>New York Yankees ML</t>
         </is>
       </c>
       <c r="E36" s="8" t="n">
-        <v>108</v>
+        <v>-106</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>0.641</v>
+        <v>0.5198</v>
       </c>
       <c r="G36" s="10" t="n">
-        <v>0.1714</v>
-      </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>⚠️ verify news</t>
-        </is>
-      </c>
+        <v>0.0252</v>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19T00:30Z</t>
+          <t>2026-07-19T23:20:00Z</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>San Diego Padres @ Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Kansas City Royals -1.5</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>163</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0.4093</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>0.0204</v>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-07-19T18:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Texas Rangers @ Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Atlanta Braves -1.5</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>170</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>0.3779</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>0.0202</v>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>San Diego Padres @ Kansas City Royals</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Kansas City Royals +1.5</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>-150</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0.6398</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Over 7.5</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>0.6228</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="H40" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T17:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers @ New York Yankees</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Under 9.0</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>117</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0.6181</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>0.2421</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-07-19T16:35:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Texas Rangers @ Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Under 9.5</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>0.6114999999999999</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <v>0.2352</v>
+      </c>
+      <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Over 7.5</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>102</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>0.6112</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>0.2347</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-07-18T23:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Minnesota Twins @ Chicago Cubs</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Over 9.0</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>0.4931</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>0.2212</v>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T18:20:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Pittsburgh Pirates @ Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Over 7.5</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>113</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>0.5631</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>0.1994</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-07-19T17:40:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>St. Louis Cardinals @ Arizona Diamondbacks</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Under 9.0</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>0.6054999999999999</v>
+      </c>
+      <c r="G46" s="10" t="n">
+        <v>0.1933</v>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T20:10:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>WNBA</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Connecticut Sun @ Phoenix Mercury</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Over 165.5</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0.6698</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>0.1796</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-07-19T23:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Portland Fire @ Minnesota Lynx</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Over 173.5</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F48" s="9" t="n">
+        <v>0.6636</v>
+      </c>
+      <c r="G48" s="10" t="n">
+        <v>0.1734</v>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Chicago Sky @ Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Over 179.5</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>0.6417</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>0.1709</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-07-19T20:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>MLB</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>New York Mets @ Philadelphia Phillies</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Under 9.0</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="F50" s="9" t="n">
+        <v>0.5860000000000001</v>
+      </c>
+      <c r="G50" s="10" t="n">
+        <v>0.1705</v>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-18T19:05:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>New York Liberty @ Indiana Fever</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Moneyline</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Indiana Fever ML</t>
         </is>
       </c>
-      <c r="E37" s="5" t="n">
-        <v>117</v>
-      </c>
-      <c r="F37" s="6" t="n">
+      <c r="E51" s="5" t="n">
+        <v>120</v>
+      </c>
+      <c r="F51" s="6" t="n">
         <v>0.6189</v>
       </c>
-      <c r="G37" s="7" t="n">
-        <v>0.1588</v>
-      </c>
-      <c r="H37" t="inlineStr">
+      <c r="G51" s="7" t="n">
+        <v>0.1653</v>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>⚠️ verify news</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>2026-07-19T00:00Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>WNBA</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Chicago Sky @ Atlanta Dream</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>Chicago Sky +10.5</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>113</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>0.6058</v>
+      </c>
+      <c r="G52" s="10" t="n">
+        <v>0.1533</v>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
+        <is>
+          <t>⚠️ verify news</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-19T20:00Z</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2884,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2320,7 +2899,7 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:17</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -2335,7 +2914,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2350,7 +2929,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2365,7 +2944,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2380,7 +2959,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -2395,7 +2974,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:54</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2410,7 +2989,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -2425,7 +3004,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2440,7 +3019,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:18</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -2455,7 +3034,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2470,7 +3049,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -2485,7 +3064,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2500,7 +3079,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -2515,7 +3094,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2530,7 +3109,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:55</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -2545,7 +3124,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2560,7 +3139,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -2575,7 +3154,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:19</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2590,7 +3169,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:20</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -2605,7 +3184,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2620,7 +3199,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:20</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -2635,7 +3214,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2650,7 +3229,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:56</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -2665,7 +3244,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2680,7 +3259,7 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -2695,7 +3274,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2710,7 +3289,7 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -2725,7 +3304,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2740,7 +3319,7 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:57</t>
+          <t>2026-07-18 22:04:21</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -2755,7 +3334,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:22</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2770,7 +3349,7 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:22</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -2785,7 +3364,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:22</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2800,7 +3379,7 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:22</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -2815,7 +3394,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:22</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2830,7 +3409,7 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
@@ -2845,7 +3424,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2860,7 +3439,7 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:58</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
@@ -2875,7 +3454,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2890,7 +3469,7 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -2905,7 +3484,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2920,7 +3499,7 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
@@ -2935,7 +3514,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:23</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2950,7 +3529,7 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
@@ -2965,7 +3544,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2980,7 +3559,7 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:13:59</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -2995,7 +3574,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3010,7 +3589,7 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
@@ -3025,7 +3604,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3040,7 +3619,7 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
@@ -3055,7 +3634,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3070,7 +3649,7 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:24</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
@@ -3085,7 +3664,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:25</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3100,7 +3679,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:00</t>
+          <t>2026-07-18 22:04:25</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -3115,7 +3694,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:25</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3130,7 +3709,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:25</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -3145,7 +3724,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:25</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3160,7 +3739,7 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
@@ -3175,7 +3754,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3190,7 +3769,7 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:01</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
@@ -3205,7 +3784,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:02</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3220,7 +3799,7 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:02</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
@@ -3235,7 +3814,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:02</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3250,7 +3829,7 @@
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:02</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
@@ -3265,7 +3844,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-18 18:14:02</t>
+          <t>2026-07-18 22:04:26</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">

</xml_diff>